<commit_message>
revies xargs, echo, read and write
</commit_message>
<xml_diff>
--- a/CSAPP/Tutorials/Attachment of Practice Problems/Practice Problem-5.8.xlsx
+++ b/CSAPP/Tutorials/Attachment of Practice Problems/Practice Problem-5.8.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Programming\Computer-Architecture\CSAPP\Tutorials\Attachment of Practice Problems\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E305DBE3-56BE-40EC-A20F-D2674F5D25D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F36B2225-3AF7-4AE9-8EA6-A8D1E9481EE8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="37">
   <si>
     <t>%rax</t>
   </si>
@@ -119,6 +119,24 @@
   <si>
     <t>read x and then multiply it with r</t>
   </si>
+  <si>
+    <t>%rsi</t>
+  </si>
+  <si>
+    <t>%rdi</t>
+  </si>
+  <si>
+    <t>Problem 5.11</t>
+  </si>
+  <si>
+    <t>See Figures in this directory.</t>
+  </si>
+  <si>
+    <t>movss -4(%rsi, %rax, 4), %xmm0</t>
+  </si>
+  <si>
+    <t>addss (%rdi, %rax, 4), %xmm0</t>
+  </si>
 </sst>
 </file>
 
@@ -208,7 +226,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -224,7 +242,16 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -234,16 +261,19 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3515,6 +3545,568 @@
         </a:p>
       </xdr:txBody>
     </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>52</xdr:row>
+      <xdr:rowOff>82550</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>590550</xdr:colOff>
+      <xdr:row>53</xdr:row>
+      <xdr:rowOff>69850</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="71" name="Rectangle: Rounded Corners 70">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{13678BA3-9196-6A20-1991-647126E7758A}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="4267200" y="15951200"/>
+          <a:ext cx="590550" cy="355600"/>
+        </a:xfrm>
+        <a:prstGeom prst="roundRect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="accent1">
+            <a:lumMod val="40000"/>
+            <a:lumOff val="60000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:ln>
+          <a:solidFill>
+            <a:schemeClr val="tx1"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="15000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:r>
+            <a:rPr lang="en-GB" sz="1400">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>add</a:t>
+          </a:r>
+          <a:endParaRPr lang="en-GB" sz="1100">
+            <a:solidFill>
+              <a:schemeClr val="tx1"/>
+            </a:solidFill>
+          </a:endParaRPr>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>260350</xdr:colOff>
+      <xdr:row>49</xdr:row>
+      <xdr:rowOff>6350</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>266700</xdr:colOff>
+      <xdr:row>52</xdr:row>
+      <xdr:rowOff>101600</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="73" name="Straight Arrow Connector 72">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8ED6B72A-F480-4B5A-1ACA-67AB24DC0BCB}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm flipH="1">
+          <a:off x="4527550" y="15036800"/>
+          <a:ext cx="6350" cy="1200150"/>
+        </a:xfrm>
+        <a:prstGeom prst="straightConnector1">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="19050">
+          <a:solidFill>
+            <a:schemeClr val="tx1"/>
+          </a:solidFill>
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>355600</xdr:colOff>
+      <xdr:row>52</xdr:row>
+      <xdr:rowOff>63500</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>336550</xdr:colOff>
+      <xdr:row>53</xdr:row>
+      <xdr:rowOff>50800</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="85" name="Rectangle: Rounded Corners 84">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{09E0C841-10A2-646C-1A62-55BAE2A261D4}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="5842000" y="15932150"/>
+          <a:ext cx="590550" cy="355600"/>
+        </a:xfrm>
+        <a:prstGeom prst="roundRect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="accent1">
+            <a:lumMod val="40000"/>
+            <a:lumOff val="60000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:ln>
+          <a:solidFill>
+            <a:schemeClr val="tx1"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="15000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:r>
+            <a:rPr lang="en-GB" sz="1400">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>load</a:t>
+          </a:r>
+          <a:endParaRPr lang="en-GB" sz="1100">
+            <a:solidFill>
+              <a:schemeClr val="tx1"/>
+            </a:solidFill>
+          </a:endParaRPr>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>539750</xdr:colOff>
+      <xdr:row>53</xdr:row>
+      <xdr:rowOff>203200</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>520700</xdr:colOff>
+      <xdr:row>54</xdr:row>
+      <xdr:rowOff>190500</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="98" name="Rectangle: Rounded Corners 97">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1344A160-B471-322D-F46B-711F7033739D}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="5416550" y="16440150"/>
+          <a:ext cx="590550" cy="355600"/>
+        </a:xfrm>
+        <a:prstGeom prst="roundRect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="accent1">
+            <a:lumMod val="40000"/>
+            <a:lumOff val="60000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:ln>
+          <a:solidFill>
+            <a:schemeClr val="tx1"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="15000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:r>
+            <a:rPr lang="en-GB" sz="1400">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>add</a:t>
+          </a:r>
+          <a:endParaRPr lang="en-GB" sz="1100">
+            <a:solidFill>
+              <a:schemeClr val="tx1"/>
+            </a:solidFill>
+          </a:endParaRPr>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>590550</xdr:colOff>
+      <xdr:row>54</xdr:row>
+      <xdr:rowOff>38100</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>571500</xdr:colOff>
+      <xdr:row>55</xdr:row>
+      <xdr:rowOff>25400</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="101" name="Rectangle: Rounded Corners 100">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{33B0DCCD-578F-0419-FC17-E734A387FDC7}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="6686550" y="16643350"/>
+          <a:ext cx="590550" cy="355600"/>
+        </a:xfrm>
+        <a:prstGeom prst="roundRect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln/>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent5"/>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="lt1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent5"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="ctr"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-GB" sz="1400">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>cmp</a:t>
+          </a:r>
+          <a:endParaRPr lang="en-GB" sz="1100">
+            <a:solidFill>
+              <a:schemeClr val="tx1"/>
+            </a:solidFill>
+          </a:endParaRPr>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>165100</xdr:colOff>
+      <xdr:row>53</xdr:row>
+      <xdr:rowOff>95250</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>171450</xdr:colOff>
+      <xdr:row>56</xdr:row>
+      <xdr:rowOff>349250</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="112" name="Straight Arrow Connector 111">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A41BC5EC-B920-225E-3FEC-91810FD31FB8}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="4432300" y="16332200"/>
+          <a:ext cx="6350" cy="1358900"/>
+        </a:xfrm>
+        <a:prstGeom prst="straightConnector1">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="19050">
+          <a:solidFill>
+            <a:schemeClr val="tx1"/>
+          </a:solidFill>
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>584200</xdr:colOff>
+      <xdr:row>55</xdr:row>
+      <xdr:rowOff>355600</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>565150</xdr:colOff>
+      <xdr:row>56</xdr:row>
+      <xdr:rowOff>342900</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="115" name="Rectangle: Rounded Corners 114">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B594F82F-1EE8-988C-B6BC-FC88EFDFC6C4}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="6680200" y="17329150"/>
+          <a:ext cx="590550" cy="355600"/>
+        </a:xfrm>
+        <a:prstGeom prst="roundRect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln/>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent5"/>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="lt1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent5"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="ctr"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-GB" sz="1400">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>jg</a:t>
+          </a:r>
+          <a:endParaRPr lang="en-GB" sz="1100">
+            <a:solidFill>
+              <a:schemeClr val="tx1"/>
+            </a:solidFill>
+          </a:endParaRPr>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>269875</xdr:colOff>
+      <xdr:row>55</xdr:row>
+      <xdr:rowOff>25400</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>276225</xdr:colOff>
+      <xdr:row>55</xdr:row>
+      <xdr:rowOff>355600</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="116" name="Straight Arrow Connector 115">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A1300809-5E1A-3685-CB53-8BD02BE0B470}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr>
+          <a:stCxn id="101" idx="2"/>
+          <a:endCxn id="115" idx="0"/>
+        </xdr:cNvCxnSpPr>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm flipH="1">
+          <a:off x="6975475" y="16998950"/>
+          <a:ext cx="6350" cy="330200"/>
+        </a:xfrm>
+        <a:prstGeom prst="straightConnector1">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="19050">
+          <a:solidFill>
+            <a:schemeClr val="tx1"/>
+          </a:solidFill>
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
@@ -3783,7 +4375,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="F8:U45"/>
+  <dimension ref="F8:U62"/>
   <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="18" width="8.7265625" style="2"/>
@@ -3814,23 +4406,23 @@
       <c r="K9" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="O9" s="9" t="s">
+      <c r="O9" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="P9" s="9"/>
-      <c r="Q9" s="9"/>
-      <c r="R9" s="9"/>
+      <c r="P9" s="11"/>
+      <c r="Q9" s="11"/>
+      <c r="R9" s="11"/>
     </row>
     <row r="10" spans="6:19" ht="30" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="M10" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="O10" s="14" t="s">
+      <c r="O10" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="P10" s="14"/>
-      <c r="Q10" s="14"/>
-      <c r="R10" s="14"/>
+      <c r="P10" s="9"/>
+      <c r="Q10" s="9"/>
+      <c r="R10" s="9"/>
       <c r="S10" s="1"/>
     </row>
     <row r="11" spans="6:19" ht="30" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
@@ -3838,12 +4430,12 @@
         <v>5</v>
       </c>
       <c r="N11" s="1"/>
-      <c r="O11" s="15" t="s">
+      <c r="O11" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="P11" s="15"/>
-      <c r="Q11" s="15"/>
-      <c r="R11" s="15"/>
+      <c r="P11" s="12"/>
+      <c r="Q11" s="12"/>
+      <c r="R11" s="12"/>
       <c r="S11" s="1" t="s">
         <v>7</v>
       </c>
@@ -3853,20 +4445,20 @@
         <v>6</v>
       </c>
       <c r="N12" s="1"/>
-      <c r="O12" s="12"/>
-      <c r="P12" s="12"/>
-      <c r="Q12" s="12"/>
-      <c r="R12" s="12"/>
+      <c r="O12" s="10"/>
+      <c r="P12" s="10"/>
+      <c r="Q12" s="10"/>
+      <c r="R12" s="10"/>
     </row>
     <row r="13" spans="6:19" ht="30" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="M13" s="4" t="s">
         <v>5</v>
       </c>
       <c r="N13" s="1"/>
-      <c r="O13" s="12"/>
-      <c r="P13" s="12"/>
-      <c r="Q13" s="12"/>
-      <c r="R13" s="12"/>
+      <c r="O13" s="10"/>
+      <c r="P13" s="10"/>
+      <c r="Q13" s="10"/>
+      <c r="R13" s="10"/>
     </row>
     <row r="14" spans="6:19" ht="30" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="M14" s="4" t="s">
@@ -4008,66 +4600,66 @@
       <c r="M32" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="Q32" s="9" t="s">
+      <c r="Q32" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="R32" s="9"/>
-      <c r="S32" s="9"/>
-      <c r="T32" s="9"/>
+      <c r="R32" s="11"/>
+      <c r="S32" s="11"/>
+      <c r="T32" s="11"/>
     </row>
-    <row r="33" spans="9:21" ht="32" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="33" spans="7:21" ht="32" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="O33" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="Q33" s="10" t="s">
+      <c r="Q33" s="13" t="s">
         <v>28</v>
       </c>
-      <c r="R33" s="10"/>
-      <c r="S33" s="10"/>
-      <c r="T33" s="10"/>
+      <c r="R33" s="13"/>
+      <c r="S33" s="13"/>
+      <c r="T33" s="13"/>
       <c r="U33" s="1"/>
     </row>
-    <row r="34" spans="9:21" ht="32" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="34" spans="7:21" ht="32" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="O34" s="4" t="s">
         <v>5</v>
       </c>
       <c r="P34" s="1"/>
-      <c r="Q34" s="11" t="s">
+      <c r="Q34" s="14" t="s">
         <v>12</v>
       </c>
-      <c r="R34" s="11"/>
-      <c r="S34" s="11"/>
-      <c r="T34" s="11"/>
+      <c r="R34" s="14"/>
+      <c r="S34" s="14"/>
+      <c r="T34" s="14"/>
       <c r="U34" s="1" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="35" spans="9:21" ht="32" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="35" spans="7:21" ht="32" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="O35" s="4" t="s">
         <v>6</v>
       </c>
       <c r="P35" s="1"/>
-      <c r="Q35" s="12"/>
-      <c r="R35" s="12"/>
-      <c r="S35" s="12"/>
-      <c r="T35" s="12"/>
+      <c r="Q35" s="10"/>
+      <c r="R35" s="10"/>
+      <c r="S35" s="10"/>
+      <c r="T35" s="10"/>
     </row>
-    <row r="36" spans="9:21" ht="32" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="36" spans="7:21" ht="32" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="O36" s="4" t="s">
         <v>5</v>
       </c>
       <c r="P36" s="1"/>
-      <c r="Q36" s="13" t="s">
+      <c r="Q36" s="15" t="s">
         <v>29</v>
       </c>
-      <c r="R36" s="13"/>
-      <c r="S36" s="13"/>
-      <c r="T36" s="13"/>
+      <c r="R36" s="15"/>
+      <c r="S36" s="15"/>
+      <c r="T36" s="15"/>
       <c r="U36" s="2" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="37" spans="9:21" ht="32" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="37" spans="7:21" ht="32" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="O37" s="4" t="s">
         <v>6</v>
       </c>
@@ -4078,7 +4670,7 @@
       <c r="T37" s="8"/>
       <c r="U37" s="1"/>
     </row>
-    <row r="38" spans="9:21" ht="32" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="38" spans="7:21" ht="32" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="O38" s="4" t="s">
         <v>6</v>
       </c>
@@ -4091,7 +4683,7 @@
       <c r="T38" s="8"/>
       <c r="U38" s="1"/>
     </row>
-    <row r="39" spans="9:21" ht="32" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="39" spans="7:21" ht="32" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="O39" s="5" t="s">
         <v>14</v>
       </c>
@@ -4102,7 +4694,7 @@
       <c r="S39" s="7"/>
       <c r="T39" s="7"/>
     </row>
-    <row r="40" spans="9:21" ht="32" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="40" spans="7:21" ht="32" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="O40" s="5" t="s">
         <v>17</v>
       </c>
@@ -4113,7 +4705,7 @@
       <c r="S40" s="7"/>
       <c r="T40" s="7"/>
     </row>
-    <row r="41" spans="9:21" ht="32" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="41" spans="7:21" ht="32" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="O41" s="5" t="s">
         <v>18</v>
       </c>
@@ -4124,14 +4716,14 @@
       <c r="S41" s="7"/>
       <c r="T41" s="7"/>
     </row>
-    <row r="42" spans="9:21" ht="32" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="42" spans="7:21" ht="32" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="O42" s="5"/>
       <c r="Q42" s="7"/>
       <c r="R42" s="7"/>
       <c r="S42" s="7"/>
       <c r="T42" s="7"/>
     </row>
-    <row r="43" spans="9:21" ht="32" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
+    <row r="43" spans="7:21" ht="32" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
       <c r="I43" s="3" t="s">
         <v>0</v>
       </c>
@@ -4152,40 +4744,101 @@
       <c r="S43" s="7"/>
       <c r="T43" s="7"/>
     </row>
-    <row r="44" spans="9:21" x14ac:dyDescent="0.35">
+    <row r="44" spans="7:21" x14ac:dyDescent="0.35">
       <c r="Q44" s="7"/>
       <c r="R44" s="7"/>
       <c r="S44" s="7"/>
       <c r="T44" s="7"/>
     </row>
-    <row r="45" spans="9:21" x14ac:dyDescent="0.35">
+    <row r="45" spans="7:21" x14ac:dyDescent="0.35">
       <c r="Q45" s="7"/>
       <c r="R45" s="7"/>
       <c r="S45" s="7"/>
       <c r="T45" s="7"/>
     </row>
+    <row r="47" spans="7:21" ht="36.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="G47" s="18" t="s">
+        <v>33</v>
+      </c>
+      <c r="H47" s="18"/>
+      <c r="K47" s="2" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="48" spans="7:21" ht="16" thickBot="1" x14ac:dyDescent="0.4"/>
+    <row r="49" spans="8:19" ht="29" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="H49" s="16" t="s">
+        <v>3</v>
+      </c>
+      <c r="I49" s="16" t="s">
+        <v>31</v>
+      </c>
+      <c r="J49" s="16" t="s">
+        <v>0</v>
+      </c>
+      <c r="K49" s="16" t="s">
+        <v>32</v>
+      </c>
+      <c r="L49" s="16" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="50" spans="8:19" ht="29" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="O50" s="16" t="s">
+        <v>5</v>
+      </c>
+      <c r="Q50" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="R50" s="8"/>
+      <c r="S50" s="8"/>
+    </row>
+    <row r="51" spans="8:19" ht="29" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="I51" s="17"/>
+      <c r="O51" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="Q51" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="R51" s="8"/>
+      <c r="S51" s="8"/>
+    </row>
+    <row r="52" spans="8:19" ht="29" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="O52" s="16"/>
+    </row>
+    <row r="53" spans="8:19" ht="29" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="O53" s="16"/>
+    </row>
+    <row r="54" spans="8:19" ht="29" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="O54" s="16"/>
+    </row>
+    <row r="55" spans="8:19" ht="29" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="O55" s="16"/>
+    </row>
+    <row r="56" spans="8:19" ht="29" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="O56" s="16"/>
+    </row>
+    <row r="57" spans="8:19" ht="29" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="O57" s="19"/>
+    </row>
+    <row r="58" spans="8:19" ht="29" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="H58" s="16" t="s">
+        <v>3</v>
+      </c>
+      <c r="J58" s="16" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59" spans="8:19" ht="29" customHeight="1" thickTop="1" x14ac:dyDescent="0.35"/>
+    <row r="60" spans="8:19" ht="29" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="61" spans="8:19" ht="29" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="62" spans="8:19" ht="29" customHeight="1" x14ac:dyDescent="0.35"/>
   </sheetData>
-  <mergeCells count="29">
-    <mergeCell ref="O16:R16"/>
-    <mergeCell ref="O15:R15"/>
-    <mergeCell ref="O10:R10"/>
-    <mergeCell ref="O12:R12"/>
-    <mergeCell ref="O9:R9"/>
-    <mergeCell ref="O11:R11"/>
-    <mergeCell ref="O14:R14"/>
-    <mergeCell ref="O13:R13"/>
-    <mergeCell ref="O23:R23"/>
-    <mergeCell ref="O17:R17"/>
-    <mergeCell ref="O18:R18"/>
-    <mergeCell ref="O19:R19"/>
-    <mergeCell ref="O20:R20"/>
-    <mergeCell ref="O21:R21"/>
-    <mergeCell ref="O22:R22"/>
-    <mergeCell ref="Q32:T32"/>
-    <mergeCell ref="Q33:T33"/>
-    <mergeCell ref="Q34:T34"/>
-    <mergeCell ref="Q35:T35"/>
-    <mergeCell ref="Q36:T36"/>
+  <mergeCells count="32">
+    <mergeCell ref="Q50:S50"/>
+    <mergeCell ref="G47:H47"/>
+    <mergeCell ref="Q51:S51"/>
     <mergeCell ref="Q42:T42"/>
     <mergeCell ref="Q43:T43"/>
     <mergeCell ref="Q44:T44"/>
@@ -4195,6 +4848,26 @@
     <mergeCell ref="Q39:T39"/>
     <mergeCell ref="Q40:T40"/>
     <mergeCell ref="Q41:T41"/>
+    <mergeCell ref="Q32:T32"/>
+    <mergeCell ref="Q33:T33"/>
+    <mergeCell ref="Q34:T34"/>
+    <mergeCell ref="Q35:T35"/>
+    <mergeCell ref="Q36:T36"/>
+    <mergeCell ref="O23:R23"/>
+    <mergeCell ref="O17:R17"/>
+    <mergeCell ref="O18:R18"/>
+    <mergeCell ref="O19:R19"/>
+    <mergeCell ref="O20:R20"/>
+    <mergeCell ref="O21:R21"/>
+    <mergeCell ref="O22:R22"/>
+    <mergeCell ref="O16:R16"/>
+    <mergeCell ref="O15:R15"/>
+    <mergeCell ref="O10:R10"/>
+    <mergeCell ref="O12:R12"/>
+    <mergeCell ref="O9:R9"/>
+    <mergeCell ref="O11:R11"/>
+    <mergeCell ref="O14:R14"/>
+    <mergeCell ref="O13:R13"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>